<commit_message>
feat(attachments): add payment attachments system with upload/download/delete via payment_id binding
- Created attachments and attachment_links tables for polymorphic file storage

- Built API routes for upload, download, delete, and list operations

- Implemented PaymentAttachments UI component with dialog and file management

- Integrated attachment UI into payments table and payments report table

- Added service layer functions in lib/attachments.ts for CRUD operations

- Created migration 20260406150000_add_attachments_base

- Added Phase 1 dictionaries (currencies, document_types, project_states, mi_dimensions)

- Storage location: Supabase Storage bucket 'payment-attachments'
</commit_message>
<xml_diff>
--- a/exports/partial_payment_matches.xlsx
+++ b/exports/partial_payment_matches.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U14"/>
+  <dimension ref="A1:V13"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="35.83203125" customWidth="1"/>
@@ -420,6 +420,7 @@
     <col min="19" max="19" width="15.83203125" customWidth="1"/>
     <col min="20" max="20" width="25.83203125" customWidth="1"/>
     <col min="21" max="21" width="20.83203125" customWidth="1"/>
+    <col min="22" max="22" width="16.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -486,37 +487,40 @@
       <c r="U1" t="str">
         <v>Job Match</v>
       </c>
+      <c r="V1" t="str">
+        <v>Has Exact Match</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>1TV Service | 1.2.1 | თბილი სახლი | 1,200.00 | USD | 15.05.2025</v>
+        <v>Biota Park | 1.1.2 | ოლიმპ ჯორჯია | 1,500.00 | USD | 29.10.2019</v>
       </c>
       <c r="B2" t="str">
-        <v>1TV Service</v>
+        <v>Biota Park</v>
       </c>
       <c r="C2" t="str">
-        <v>თბილი სახლი</v>
+        <v>ოლიმპ ჯორჯია</v>
       </c>
       <c r="D2" t="str">
-        <v>204976179</v>
+        <v>405231011</v>
       </c>
       <c r="E2" t="str">
-        <v>1.2.1</v>
+        <v>1.1.2</v>
       </c>
       <c r="F2" t="str">
-        <v>შემოსავალი MEP დანადგარების რეალიზაციიდან</v>
+        <v>შემოსავალი ლიფტების სერვისიდან - გეგმიური</v>
       </c>
       <c r="G2" t="str">
         <v>USD</v>
       </c>
       <c r="H2">
-        <v>1200</v>
+        <v>1500</v>
       </c>
       <c r="I2" t="str">
-        <v>15/05/2025</v>
+        <v>29/10/2019</v>
       </c>
       <c r="J2" t="str">
-        <v>5cfaed_5f_2e2feb</v>
+        <v>e17787_1d_b93431</v>
       </c>
       <c r="K2" t="b">
         <v>1</v>
@@ -534,54 +538,57 @@
         <v>შემოსავალი ლიფტების სერვისიდან - გეგმიური</v>
       </c>
       <c r="P2" t="str">
-        <v>USD</v>
+        <v>GEL</v>
       </c>
       <c r="Q2" t="str">
         <v>(none)</v>
       </c>
       <c r="R2" t="str">
+        <v>OK</v>
+      </c>
+      <c r="S2" t="str">
         <v>MISMATCH</v>
       </c>
-      <c r="S2" t="str">
-        <v>OK</v>
-      </c>
       <c r="T2" t="str">
         <v>OK</v>
       </c>
       <c r="U2" t="str">
         <v>OK</v>
+      </c>
+      <c r="V2" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Biota Park | 1.1.2 | ოლიმპ ჯორჯია | 1,500.00 | USD | 29.10.2019</v>
+        <v>Card System Adaptation | 1.1.3 | ორბი ჯგუფი ბათუმი | 99,619.50 | USD | 16.06.2025</v>
       </c>
       <c r="B3" t="str">
-        <v>Biota Park</v>
+        <v>Card System Adaptation</v>
       </c>
       <c r="C3" t="str">
-        <v>ოლიმპ ჯორჯია</v>
+        <v>ორბი ჯგუფი ბათუმი</v>
       </c>
       <c r="D3" t="str">
-        <v>405231011</v>
+        <v>445468798</v>
       </c>
       <c r="E3" t="str">
-        <v>1.1.2</v>
+        <v>1.1.3</v>
       </c>
       <c r="F3" t="str">
-        <v>შემოსავალი ლიფტების სერვისიდან - გეგმიური</v>
+        <v>შემოსავალი ლიფტების სერვისიდან - არაგეგმიური</v>
       </c>
       <c r="G3" t="str">
         <v>USD</v>
       </c>
       <c r="H3">
-        <v>1500</v>
+        <v>99619.5</v>
       </c>
       <c r="I3" t="str">
-        <v>29/10/2019</v>
+        <v>16/06/2025</v>
       </c>
       <c r="J3" t="str">
-        <v>e17787_1d_b93431</v>
+        <v>ef4884_75_8194a0</v>
       </c>
       <c r="K3" t="b">
         <v>1</v>
@@ -593,60 +600,63 @@
         <v>0</v>
       </c>
       <c r="N3" t="str">
-        <v>1.1.2</v>
+        <v>1.1.1</v>
       </c>
       <c r="O3" t="str">
-        <v>შემოსავალი ლიფტების სერვისიდან - გეგმიური</v>
+        <v>შემოსავალი ლიფტების რეალიზაციიდან</v>
       </c>
       <c r="P3" t="str">
-        <v>GEL</v>
+        <v>USD</v>
       </c>
       <c r="Q3" t="str">
         <v>(none)</v>
       </c>
       <c r="R3" t="str">
-        <v>OK</v>
+        <v>MISMATCH</v>
       </c>
       <c r="S3" t="str">
-        <v>MISMATCH</v>
+        <v>OK</v>
       </c>
       <c r="T3" t="str">
         <v>OK</v>
       </c>
       <c r="U3" t="str">
         <v>OK</v>
+      </c>
+      <c r="V3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Card System Adaptation | 1.1.3 | ორბი ჯგუფი ბათუმი | 99,619.50 | USD | 16.06.2025</v>
+        <v>Central Office | 1.2.1 | თბილისი ცენტრალი | 364,528.00 | USD | 28.03.2023</v>
       </c>
       <c r="B4" t="str">
-        <v>Card System Adaptation</v>
+        <v>Central Office</v>
       </c>
       <c r="C4" t="str">
-        <v>ორბი ჯგუფი ბათუმი</v>
+        <v>თბილისი ცენტრალი</v>
       </c>
       <c r="D4" t="str">
-        <v>445468798</v>
+        <v>205129653</v>
       </c>
       <c r="E4" t="str">
-        <v>1.1.3</v>
+        <v>1.2.1</v>
       </c>
       <c r="F4" t="str">
-        <v>შემოსავალი ლიფტების სერვისიდან - არაგეგმიური</v>
+        <v>შემოსავალი MEP დანადგარების რეალიზაციიდან</v>
       </c>
       <c r="G4" t="str">
         <v>USD</v>
       </c>
       <c r="H4">
-        <v>99619.5</v>
+        <v>364528</v>
       </c>
       <c r="I4" t="str">
-        <v>16/06/2025</v>
+        <v>28/03/2023</v>
       </c>
       <c r="J4" t="str">
-        <v>ef4884_75_8194a0</v>
+        <v>fe3d6d_6b_84fc7e</v>
       </c>
       <c r="K4" t="b">
         <v>1</v>
@@ -655,13 +665,13 @@
         <v>0</v>
       </c>
       <c r="M4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N4" t="str">
-        <v>1.1.1</v>
+        <v>1.2.1</v>
       </c>
       <c r="O4" t="str">
-        <v>შემოსავალი ლიფტების რეალიზაციიდან</v>
+        <v>შემოსავალი MEP დანადგარების რეალიზაციიდან</v>
       </c>
       <c r="P4" t="str">
         <v>USD</v>
@@ -670,48 +680,51 @@
         <v>(none)</v>
       </c>
       <c r="R4" t="str">
-        <v>MISMATCH</v>
+        <v>OK</v>
       </c>
       <c r="S4" t="str">
         <v>OK</v>
       </c>
       <c r="T4" t="str">
-        <v>OK</v>
+        <v>MISMATCH (true vs false)</v>
       </c>
       <c r="U4" t="str">
         <v>OK</v>
+      </c>
+      <c r="V4" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Central Office | 1.2.1 | თბილისი ცენტრალი | 364,528.00 | USD | 28.03.2023</v>
+        <v>Digomi Trade Center | 1.1.2 | ავტოტრანსპორტი 91 | 750.00 | USD | 01.01.2024</v>
       </c>
       <c r="B5" t="str">
-        <v>Central Office</v>
+        <v>Digomi Trade Center</v>
       </c>
       <c r="C5" t="str">
-        <v>თბილისი ცენტრალი</v>
+        <v>ავტოტრანსპორტი 91</v>
       </c>
       <c r="D5" t="str">
-        <v>205129653</v>
+        <v>212670091</v>
       </c>
       <c r="E5" t="str">
-        <v>1.2.1</v>
+        <v>1.1.2</v>
       </c>
       <c r="F5" t="str">
-        <v>შემოსავალი MEP დანადგარების რეალიზაციიდან</v>
+        <v>შემოსავალი ლიფტების სერვისიდან - გეგმიური</v>
       </c>
       <c r="G5" t="str">
         <v>USD</v>
       </c>
       <c r="H5">
-        <v>364528</v>
+        <v>750</v>
       </c>
       <c r="I5" t="str">
-        <v>28/03/2023</v>
+        <v>01/01/2024</v>
       </c>
       <c r="J5" t="str">
-        <v>fe3d6d_6b_84fc7e</v>
+        <v>0c4450_19_8e76c4</v>
       </c>
       <c r="K5" t="b">
         <v>1</v>
@@ -720,16 +733,16 @@
         <v>0</v>
       </c>
       <c r="M5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N5" t="str">
-        <v>1.2.1</v>
+        <v>1.1.2</v>
       </c>
       <c r="O5" t="str">
-        <v>შემოსავალი MEP დანადგარების რეალიზაციიდან</v>
+        <v>შემოსავალი ლიფტების სერვისიდან - გეგმიური</v>
       </c>
       <c r="P5" t="str">
-        <v>USD</v>
+        <v>GEL</v>
       </c>
       <c r="Q5" t="str">
         <v>(none)</v>
@@ -738,27 +751,30 @@
         <v>OK</v>
       </c>
       <c r="S5" t="str">
-        <v>OK</v>
+        <v>MISMATCH</v>
       </c>
       <c r="T5" t="str">
-        <v>MISMATCH (true vs false)</v>
+        <v>OK</v>
       </c>
       <c r="U5" t="str">
         <v>OK</v>
+      </c>
+      <c r="V5" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Digomi Trade Center | 1.1.2 | ავტოტრანსპორტი 91 | 750.00 | USD | 01.01.2024</v>
+        <v>Green Cape | 1.1.2 | ელტური-2008 | 1,000.00 | USD | 26.12.2018</v>
       </c>
       <c r="B6" t="str">
-        <v>Digomi Trade Center</v>
+        <v>Green Cape</v>
       </c>
       <c r="C6" t="str">
-        <v>ავტოტრანსპორტი 91</v>
+        <v>ელტური-2008</v>
       </c>
       <c r="D6" t="str">
-        <v>212670091</v>
+        <v>248434038</v>
       </c>
       <c r="E6" t="str">
         <v>1.1.2</v>
@@ -770,13 +786,13 @@
         <v>USD</v>
       </c>
       <c r="H6">
-        <v>750</v>
+        <v>1000</v>
       </c>
       <c r="I6" t="str">
-        <v>01/01/2024</v>
+        <v>26/12/2018</v>
       </c>
       <c r="J6" t="str">
-        <v>0c4450_19_8e76c4</v>
+        <v>92af62_92_a5264d</v>
       </c>
       <c r="K6" t="b">
         <v>1</v>
@@ -810,38 +826,41 @@
       </c>
       <c r="U6" t="str">
         <v>OK</v>
+      </c>
+      <c r="V6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Green Cape | 1.1.2 | ელტური-2008 | 1,000.00 | USD | 26.12.2018</v>
+        <v>Kvareli VRV | 1.2.1 | ინდეკო სი ემ  | 254,269.84 | USD | 01.11.2022</v>
       </c>
       <c r="B7" t="str">
-        <v>Green Cape</v>
+        <v>Kvareli VRV</v>
       </c>
       <c r="C7" t="str">
-        <v>ელტური-2008</v>
+        <v xml:space="preserve">ინდეკო სი ემ </v>
       </c>
       <c r="D7" t="str">
-        <v>248434038</v>
+        <v>405508339</v>
       </c>
       <c r="E7" t="str">
-        <v>1.1.2</v>
+        <v>1.2.1</v>
       </c>
       <c r="F7" t="str">
-        <v>შემოსავალი ლიფტების სერვისიდან - გეგმიური</v>
+        <v>შემოსავალი MEP დანადგარების რეალიზაციიდან</v>
       </c>
       <c r="G7" t="str">
         <v>USD</v>
       </c>
       <c r="H7">
-        <v>1000</v>
+        <v>254269.84</v>
       </c>
       <c r="I7" t="str">
-        <v>26/12/2018</v>
+        <v>01/11/2022</v>
       </c>
       <c r="J7" t="str">
-        <v>92af62_92_a5264d</v>
+        <v>7d895d_da_a0efeb</v>
       </c>
       <c r="K7" t="b">
         <v>1</v>
@@ -850,16 +869,16 @@
         <v>0</v>
       </c>
       <c r="M7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N7" t="str">
-        <v>1.1.2</v>
+        <v>1.2.1</v>
       </c>
       <c r="O7" t="str">
-        <v>შემოსავალი ლიფტების სერვისიდან - გეგმიური</v>
+        <v>შემოსავალი MEP დანადგარების რეალიზაციიდან</v>
       </c>
       <c r="P7" t="str">
-        <v>GEL</v>
+        <v>USD</v>
       </c>
       <c r="Q7" t="str">
         <v>(none)</v>
@@ -868,13 +887,16 @@
         <v>OK</v>
       </c>
       <c r="S7" t="str">
-        <v>MISMATCH</v>
+        <v>OK</v>
       </c>
       <c r="T7" t="str">
-        <v>OK</v>
+        <v>MISMATCH (true vs false)</v>
       </c>
       <c r="U7" t="str">
         <v>OK</v>
+      </c>
+      <c r="V7" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -906,7 +928,7 @@
         <v>01/11/2022</v>
       </c>
       <c r="J8" t="str">
-        <v>7d895d_da_a0efeb</v>
+        <v>bb12dc_ab_82181a</v>
       </c>
       <c r="K8" t="b">
         <v>1</v>
@@ -918,10 +940,10 @@
         <v>1</v>
       </c>
       <c r="N8" t="str">
-        <v>1.2.1</v>
+        <v>1.2.3</v>
       </c>
       <c r="O8" t="str">
-        <v>შემოსავალი MEP დანადგარების რეალიზაციიდან</v>
+        <v>შემოსავალი MEP დანადგარების სერვისიდან - არაგეგმიური</v>
       </c>
       <c r="P8" t="str">
         <v>USD</v>
@@ -930,7 +952,7 @@
         <v>(none)</v>
       </c>
       <c r="R8" t="str">
-        <v>OK</v>
+        <v>MISMATCH</v>
       </c>
       <c r="S8" t="str">
         <v>OK</v>
@@ -940,20 +962,23 @@
       </c>
       <c r="U8" t="str">
         <v>OK</v>
+      </c>
+      <c r="V8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Kvareli VRV | 1.2.1 | ინდეკო სი ემ  | 254,269.84 | USD | 01.11.2022</v>
+        <v>Multisplits PHS | 1.2.1 | ნუცუბიძე | 387,000.00 | USD | 01.05.2023</v>
       </c>
       <c r="B9" t="str">
-        <v>Kvareli VRV</v>
+        <v>Multisplits PHS</v>
       </c>
       <c r="C9" t="str">
-        <v xml:space="preserve">ინდეკო სი ემ </v>
+        <v>ნუცუბიძე</v>
       </c>
       <c r="D9" t="str">
-        <v>405508339</v>
+        <v>405387861</v>
       </c>
       <c r="E9" t="str">
         <v>1.2.1</v>
@@ -965,13 +990,13 @@
         <v>USD</v>
       </c>
       <c r="H9">
-        <v>254269.84</v>
+        <v>387000</v>
       </c>
       <c r="I9" t="str">
-        <v>01/11/2022</v>
+        <v>01/05/2023</v>
       </c>
       <c r="J9" t="str">
-        <v>bb12dc_ab_82181a</v>
+        <v>d3bac9_ec_a304c3</v>
       </c>
       <c r="K9" t="b">
         <v>1</v>
@@ -983,10 +1008,10 @@
         <v>1</v>
       </c>
       <c r="N9" t="str">
-        <v>1.2.3</v>
+        <v>1.2.1</v>
       </c>
       <c r="O9" t="str">
-        <v>შემოსავალი MEP დანადგარების სერვისიდან - არაგეგმიური</v>
+        <v>შემოსავალი MEP დანადგარების რეალიზაციიდან</v>
       </c>
       <c r="P9" t="str">
         <v>USD</v>
@@ -995,7 +1020,7 @@
         <v>(none)</v>
       </c>
       <c r="R9" t="str">
-        <v>MISMATCH</v>
+        <v>OK</v>
       </c>
       <c r="S9" t="str">
         <v>OK</v>
@@ -1005,38 +1030,41 @@
       </c>
       <c r="U9" t="str">
         <v>OK</v>
+      </c>
+      <c r="V9" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Multisplits PHS | 1.2.1 | ნუცუბიძე | 387,000.00 | USD | 01.05.2023</v>
+        <v>Sololaki | 1.1.2 | კანოპუსი | 250.00 | USD | 31.10.2019</v>
       </c>
       <c r="B10" t="str">
-        <v>Multisplits PHS</v>
+        <v>Sololaki</v>
       </c>
       <c r="C10" t="str">
-        <v>ნუცუბიძე</v>
+        <v>კანოპუსი</v>
       </c>
       <c r="D10" t="str">
-        <v>405387861</v>
+        <v>405229881</v>
       </c>
       <c r="E10" t="str">
-        <v>1.2.1</v>
+        <v>1.1.2</v>
       </c>
       <c r="F10" t="str">
-        <v>შემოსავალი MEP დანადგარების რეალიზაციიდან</v>
+        <v>შემოსავალი ლიფტების სერვისიდან - გეგმიური</v>
       </c>
       <c r="G10" t="str">
         <v>USD</v>
       </c>
       <c r="H10">
-        <v>387000</v>
+        <v>250</v>
       </c>
       <c r="I10" t="str">
-        <v>01/05/2023</v>
+        <v>31/10/2019</v>
       </c>
       <c r="J10" t="str">
-        <v>d3bac9_ec_a304c3</v>
+        <v>072ad9_6e_1f47b4</v>
       </c>
       <c r="K10" t="b">
         <v>1</v>
@@ -1045,16 +1073,16 @@
         <v>0</v>
       </c>
       <c r="M10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N10" t="str">
-        <v>1.2.1</v>
+        <v>1.1.2</v>
       </c>
       <c r="O10" t="str">
-        <v>შემოსავალი MEP დანადგარების რეალიზაციიდან</v>
+        <v>შემოსავალი ლიფტების სერვისიდან - გეგმიური</v>
       </c>
       <c r="P10" t="str">
-        <v>USD</v>
+        <v>GEL</v>
       </c>
       <c r="Q10" t="str">
         <v>(none)</v>
@@ -1063,45 +1091,48 @@
         <v>OK</v>
       </c>
       <c r="S10" t="str">
-        <v>OK</v>
+        <v>MISMATCH</v>
       </c>
       <c r="T10" t="str">
-        <v>MISMATCH (true vs false)</v>
+        <v>OK</v>
       </c>
       <c r="U10" t="str">
         <v>OK</v>
+      </c>
+      <c r="V10" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Sololaki | 1.1.2 | კანოპუსი | 250.00 | USD | 31.10.2019</v>
+        <v>Tegeta Chiller | 1.2.1 | თეგეტა მოტორსი | 257,240.00 | EUR | 26.06.2024</v>
       </c>
       <c r="B11" t="str">
-        <v>Sololaki</v>
+        <v>Tegeta Chiller</v>
       </c>
       <c r="C11" t="str">
-        <v>კანოპუსი</v>
+        <v>თეგეტა მოტორსი</v>
       </c>
       <c r="D11" t="str">
-        <v>405229881</v>
+        <v>202177205</v>
       </c>
       <c r="E11" t="str">
-        <v>1.1.2</v>
+        <v>1.2.1</v>
       </c>
       <c r="F11" t="str">
-        <v>შემოსავალი ლიფტების სერვისიდან - გეგმიური</v>
+        <v>შემოსავალი MEP დანადგარების რეალიზაციიდან</v>
       </c>
       <c r="G11" t="str">
-        <v>USD</v>
+        <v>EUR</v>
       </c>
       <c r="H11">
-        <v>250</v>
+        <v>257240</v>
       </c>
       <c r="I11" t="str">
-        <v>31/10/2019</v>
+        <v>26/06/2024</v>
       </c>
       <c r="J11" t="str">
-        <v>072ad9_6e_1f47b4</v>
+        <v>ee23f3_ff_8d3bba</v>
       </c>
       <c r="K11" t="b">
         <v>1</v>
@@ -1113,10 +1144,10 @@
         <v>0</v>
       </c>
       <c r="N11" t="str">
-        <v>1.1.2</v>
+        <v>1.2.1</v>
       </c>
       <c r="O11" t="str">
-        <v>შემოსავალი ლიფტების სერვისიდან - გეგმიური</v>
+        <v>შემოსავალი MEP დანადგარების რეალიზაციიდან</v>
       </c>
       <c r="P11" t="str">
         <v>GEL</v>
@@ -1135,38 +1166,41 @@
       </c>
       <c r="U11" t="str">
         <v>OK</v>
+      </c>
+      <c r="V11" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Tegeta Chiller | 1.2.1 | თეგეტა მოტორსი | 257,240.00 | EUR | 26.06.2024</v>
+        <v>V-JEO Restaurant Service | 1.1.2 | ვ-ჯეო რესტორნები | 500.00 | GEL | 30.04.2024</v>
       </c>
       <c r="B12" t="str">
-        <v>Tegeta Chiller</v>
+        <v>V-JEO Restaurant Service</v>
       </c>
       <c r="C12" t="str">
-        <v>თეგეტა მოტორსი</v>
+        <v>ვ-ჯეო რესტორნები</v>
       </c>
       <c r="D12" t="str">
-        <v>202177205</v>
+        <v>405404076</v>
       </c>
       <c r="E12" t="str">
-        <v>1.2.1</v>
+        <v>1.1.2</v>
       </c>
       <c r="F12" t="str">
-        <v>შემოსავალი MEP დანადგარების რეალიზაციიდან</v>
+        <v>შემოსავალი ლიფტების სერვისიდან - გეგმიური</v>
       </c>
       <c r="G12" t="str">
-        <v>EUR</v>
+        <v>GEL</v>
       </c>
       <c r="H12">
-        <v>257240</v>
+        <v>500</v>
       </c>
       <c r="I12" t="str">
-        <v>26/06/2024</v>
+        <v>30/04/2024</v>
       </c>
       <c r="J12" t="str">
-        <v>ee23f3_ff_8d3bba</v>
+        <v>db0061_9a_d62619</v>
       </c>
       <c r="K12" t="b">
         <v>1</v>
@@ -1178,10 +1212,10 @@
         <v>0</v>
       </c>
       <c r="N12" t="str">
-        <v>1.2.1</v>
+        <v>1.1.3</v>
       </c>
       <c r="O12" t="str">
-        <v>შემოსავალი MEP დანადგარების რეალიზაციიდან</v>
+        <v>შემოსავალი ლიფტების სერვისიდან - არაგეგმიური</v>
       </c>
       <c r="P12" t="str">
         <v>GEL</v>
@@ -1190,30 +1224,33 @@
         <v>(none)</v>
       </c>
       <c r="R12" t="str">
-        <v>OK</v>
+        <v>MISMATCH</v>
       </c>
       <c r="S12" t="str">
-        <v>MISMATCH</v>
+        <v>OK</v>
       </c>
       <c r="T12" t="str">
         <v>OK</v>
       </c>
       <c r="U12" t="str">
         <v>OK</v>
+      </c>
+      <c r="V12" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>V-JEO Restaurant Service | 1.1.2 | ვ-ჯეო რესტორნები | 500.00 | GEL | 30.04.2024</v>
+        <v>Varketili | 1.1.2 | გიოკაპიტალი | 150.00 | USD | 16.09.2019</v>
       </c>
       <c r="B13" t="str">
-        <v>V-JEO Restaurant Service</v>
+        <v>Varketili</v>
       </c>
       <c r="C13" t="str">
-        <v>ვ-ჯეო რესტორნები</v>
+        <v>გიოკაპიტალი</v>
       </c>
       <c r="D13" t="str">
-        <v>405404076</v>
+        <v>406155841</v>
       </c>
       <c r="E13" t="str">
         <v>1.1.2</v>
@@ -1222,16 +1259,16 @@
         <v>შემოსავალი ლიფტების სერვისიდან - გეგმიური</v>
       </c>
       <c r="G13" t="str">
-        <v>GEL</v>
+        <v>USD</v>
       </c>
       <c r="H13">
-        <v>500</v>
+        <v>150</v>
       </c>
       <c r="I13" t="str">
-        <v>30/04/2024</v>
+        <v>16/09/2019</v>
       </c>
       <c r="J13" t="str">
-        <v>db0061_9a_d62619</v>
+        <v>8509d8_06_e9eaef</v>
       </c>
       <c r="K13" t="b">
         <v>1</v>
@@ -1243,10 +1280,10 @@
         <v>0</v>
       </c>
       <c r="N13" t="str">
-        <v>1.1.3</v>
+        <v>1.1.2</v>
       </c>
       <c r="O13" t="str">
-        <v>შემოსავალი ლიფტების სერვისიდან - არაგეგმიური</v>
+        <v>შემოსავალი ლიფტების სერვისიდან - გეგმიური</v>
       </c>
       <c r="P13" t="str">
         <v>GEL</v>
@@ -1255,86 +1292,24 @@
         <v>(none)</v>
       </c>
       <c r="R13" t="str">
+        <v>OK</v>
+      </c>
+      <c r="S13" t="str">
         <v>MISMATCH</v>
       </c>
-      <c r="S13" t="str">
-        <v>OK</v>
-      </c>
       <c r="T13" t="str">
         <v>OK</v>
       </c>
       <c r="U13" t="str">
         <v>OK</v>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Varketili | 1.1.2 | გიოკაპიტალი | 150.00 | USD | 16.09.2019</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Varketili</v>
-      </c>
-      <c r="C14" t="str">
-        <v>გიოკაპიტალი</v>
-      </c>
-      <c r="D14" t="str">
-        <v>406155841</v>
-      </c>
-      <c r="E14" t="str">
-        <v>1.1.2</v>
-      </c>
-      <c r="F14" t="str">
-        <v>შემოსავალი ლიფტების სერვისიდან - გეგმიური</v>
-      </c>
-      <c r="G14" t="str">
-        <v>USD</v>
-      </c>
-      <c r="H14">
-        <v>150</v>
-      </c>
-      <c r="I14" t="str">
-        <v>16/09/2019</v>
-      </c>
-      <c r="J14" t="str">
-        <v>8509d8_06_e9eaef</v>
-      </c>
-      <c r="K14" t="b">
-        <v>1</v>
-      </c>
-      <c r="L14" t="b">
-        <v>0</v>
-      </c>
-      <c r="M14" t="b">
-        <v>0</v>
-      </c>
-      <c r="N14" t="str">
-        <v>1.1.2</v>
-      </c>
-      <c r="O14" t="str">
-        <v>შემოსავალი ლიფტების სერვისიდან - გეგმიური</v>
-      </c>
-      <c r="P14" t="str">
-        <v>GEL</v>
-      </c>
-      <c r="Q14" t="str">
-        <v>(none)</v>
-      </c>
-      <c r="R14" t="str">
-        <v>OK</v>
-      </c>
-      <c r="S14" t="str">
-        <v>MISMATCH</v>
-      </c>
-      <c r="T14" t="str">
-        <v>OK</v>
-      </c>
-      <c r="U14" t="str">
-        <v>OK</v>
+      <c r="V13" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:U14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>